<commit_message>
Added other remaining class files.
</commit_message>
<xml_diff>
--- a/L I S 440/Lectures/Week 3/JeffNyhoff_XLdemo_AlejandroDeLaTorre.xlsx
+++ b/L I S 440/Lectures/Week 3/JeffNyhoff_XLdemo_AlejandroDeLaTorre.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffn\Box\UW\UWiSchool\Fall2023\LIS351\wk13\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwprod-my.sharepoint.com/personal/adelatorre2_wisc_edu/Documents/Coursework/L I S 440/Lectures/Week 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B61487E8-314A-4FEC-A67D-CB0B1240011D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{B61487E8-314A-4FEC-A67D-CB0B1240011D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2392A89-77A1-47A3-8D13-FF6ADC59B885}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="838" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22920" windowHeight="13800" tabRatio="838" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blank" sheetId="18" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -54,14 +54,21 @@
   <si>
     <t xml:space="preserve">Next: </t>
   </si>
+  <si>
+    <t>Percent:</t>
+  </si>
+  <si>
+    <t>Total:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -147,9 +154,9 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -467,31 +474,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L18"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B1" s="4"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="9"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="4"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
     </row>
-    <row r="18" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="12:12" x14ac:dyDescent="0.2">
       <c r="L18" s="4"/>
     </row>
   </sheetData>
@@ -505,22 +512,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1">
         <v>2023</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B2" s="1">
         <v>2024</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>0</v>
       </c>
@@ -536,30 +543,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:C26"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.21875" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1">
         <v>2024</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B2" s="1">
         <f>A1</f>
         <v>2024</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C3" s="6"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="5"/>
       <c r="B4" s="2"/>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>0</v>
       </c>
@@ -575,9 +582,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>3</v>
       </c>
@@ -587,18 +594,18 @@
       <c r="E1" s="1"/>
       <c r="F1" s="7"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="10">
         <f>B1+1</f>
         <v>2024</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="8"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E3" s="1"/>
       <c r="F3" s="7"/>
     </row>
@@ -612,31 +619,31 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC4FB22E-1E27-44AD-8C68-5EF0A74841ED}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="6">
         <f ca="1">YEAR( TODAY()  )</f>
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="7"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="10">
         <f ca="1">B1+1</f>
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="8"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E3" s="1"/>
       <c r="F3" s="7"/>
     </row>
@@ -649,28 +656,41 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDDA2D52-FC15-4494-90D3-9E761CD28A7A}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10">
+      <c r="B1" s="12">
         <v>20.440000000000001</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="12"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="11">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10">
-        <f>B1*0.25</f>
-        <v>5.1100000000000003</v>
+      <c r="B3" s="12">
+        <f>B1*B2</f>
+        <v>4.4968000000000004</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="12">
+        <f>B1+B3</f>
+        <v>24.936800000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>